<commit_message>
Merge 13/10 + coleta parcial do robo (76 de 91 insumos) - para continuar no EPMUDA 428
</commit_message>
<xml_diff>
--- a/FNDE/Centro Oeste/Fornecedores/FNDE_EPI_UNIFORME.xlsx
+++ b/FNDE/Centro Oeste/Fornecedores/FNDE_EPI_UNIFORME.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1973,6 +1973,456 @@
       <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Empresas_Pesquisa_SEAD_GO_Limpeza_1.xlsx (aba Preço aberto no site)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Bauru</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>EPI'S ONLINE COMERCIO LTDA (EPI's Online)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>22.712.006/0001-24</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4642-7/02 (secundário)</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.episonline.com.br</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.episonline.com.br</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.episonline.com.br | https://publica.cnpj.ws/cnpj/22712006000124</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Itapuí</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>L.R. COMERCIO DE SUPRIMENTOS LTDA (Fast EPIs)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>22.966.860/0001-17</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>4642-7/02 (principal); 4647-8/01 (secundário); 4649-4/08 (secundário); 4651-6/02 (secundário); 4672-9/00 (secundário)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fastepis.com.br</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fastepis.com.br</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fastepis.com.br | https://publica.cnpj.ws/cnpj/22966860000117</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Campo Grande</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>COMERCIAL DE REFRIGERACAO PANAN OESTE LTDA (Panan)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>15.448.996/0001-70</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>4665-6/00 (principal); 4614-1/00 (secundário); 4649-4/01 (secundário); 4649-4/04 (secundário)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.panan.com.br</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.panan.com.br</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.panan.com.br | https://publica.cnpj.ws/cnpj/15448996000170</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Franca</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>PALACIO DAS FERRAMENTAS E PARAFUSOS LTDA (Palácio das Ferramentas)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>68.422.419/0001-75</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>4661-3/00 (secundário); 4662-1/00 (secundário); 4663-0/00 (secundário); 4672-9/00 (secundário)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>https://palaciodasferramentas.com.br</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>https://palaciodasferramentas.com.br</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>https://palaciodasferramentas.com.br | https://publica.cnpj.ws/cnpj/68422419000175</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Mineiros</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>VALTER RAMOS LTDA (Goiás Ferramentas)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>09.497.806/0001-01</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>4672-9/00 (principal); 4661-3/00 (secundário)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goiasferramentas.com.br</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goiasferramentas.com.br</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.goiasferramentas.com.br | https://publica.cnpj.ws/cnpj/09497806000101</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Mineiros</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>MARCHIO MATERIAIS DE CONSTRUCAO E TRANSPORTE LTDA (Marchio)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>21.438.421/0004-11</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>4679-6/99 (principal)</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marchio.com</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marchio.com</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marchio.com | https://publica.cnpj.ws/cnpj/21438421000411</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Extrema</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>CALCADOS PARA TRABALHAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Calçados para Trabalhar)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>30.420.742/0002-18</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>4642-7/02 (secundário)</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.calcadosparatrabalhar.com.br</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.calcadosparatrabalhar.com.br</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.calcadosparatrabalhar.com.br | https://publica.cnpj.ws/cnpj/30420742000218</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Santo André</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>NOVA LIMP COMERCIO DE EMBALAGENS E DESCARTAVEIS LTDA (Nova Limp)</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>04.681.311/0001-14</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>4693-1/00 (principal); 4649-4/99 (secundário); 4686-9/02 (secundário)</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.novalimp.com.br</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.novalimp.com.br</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.novalimp.com.br | https://publica.cnpj.ws/cnpj/04681311000114</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>MAK-FRIGO REFRIGERACAO LTDA (Frigo)</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>57.885.329/0003-66</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>4649-4/01 (secundário); 4649-4/99 (secundário); 4665-6/00 (secundário)</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.frigo.com.br</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>https://www.frigo.com.br</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Incluído em 13/10/2026 a partir da entrega do William; razão social, UF, cidade e CNAE conferidos na Receita (publica.cnpj.ws). Demais campos não verificados.</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frigo.com.br | https://publica.cnpj.ws/cnpj/57885329000366</t>
         </is>
       </c>
     </row>
@@ -2034,6 +2484,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3144,7 +3603,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3226,7 +3684,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>

</xml_diff>